<commit_message>
#7 1 Board BOM Price Update
</commit_message>
<xml_diff>
--- a/Design Files/Xponent-tech/BOM/eSpark-BOM-Xponent-tech.xlsx
+++ b/Design Files/Xponent-tech/BOM/eSpark-BOM-Xponent-tech.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1589" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1588" uniqueCount="318">
   <si>
     <t>Component list</t>
   </si>
@@ -1446,7 +1446,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1684,6 +1684,44 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="22" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2135,7 +2173,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R61"/>
+  <dimension ref="A1:R60"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
@@ -4934,69 +4972,69 @@
     </row>
     <row r="59" spans="1:18" s="68" customFormat="1" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="66"/>
-      <c r="B59" s="47">
+      <c r="B59" s="87">
         <f t="shared" si="0"/>
         <v>50</v>
       </c>
-      <c r="C59" s="54" t="s">
+      <c r="C59" s="88" t="s">
         <v>312</v>
       </c>
-      <c r="D59" s="51" t="s">
+      <c r="D59" s="59" t="s">
         <v>67</v>
       </c>
-      <c r="E59" s="51" t="s">
+      <c r="E59" s="59" t="s">
         <v>118</v>
       </c>
-      <c r="F59" s="51" t="s">
+      <c r="F59" s="59" t="s">
         <v>130</v>
       </c>
-      <c r="G59" s="51" t="s">
+      <c r="G59" s="59" t="s">
         <v>180</v>
       </c>
-      <c r="H59" s="51" t="s">
+      <c r="H59" s="59" t="s">
         <v>199</v>
       </c>
-      <c r="I59" s="51" t="s">
-        <v>301</v>
-      </c>
-      <c r="J59" s="51" t="s">
+      <c r="I59" s="59" t="s">
+        <v>301</v>
+      </c>
+      <c r="J59" s="59" t="s">
         <v>299</v>
       </c>
-      <c r="K59" s="51" t="s">
-        <v>301</v>
-      </c>
-      <c r="L59" s="51">
+      <c r="K59" s="59" t="s">
+        <v>301</v>
+      </c>
+      <c r="L59" s="59">
         <v>3</v>
       </c>
-      <c r="M59" s="51">
+      <c r="M59" s="59">
         <v>5</v>
       </c>
-      <c r="N59" s="64" t="s">
-        <v>300</v>
-      </c>
-      <c r="O59" s="52">
+      <c r="N59" s="89" t="s">
+        <v>300</v>
+      </c>
+      <c r="O59" s="90">
         <v>0.1139</v>
       </c>
-      <c r="P59" s="52">
+      <c r="P59" s="90">
         <f t="shared" ref="P59" si="24">O59*M59</f>
         <v>0.56950000000000001</v>
       </c>
-      <c r="Q59" s="51"/>
-      <c r="R59" s="39"/>
+      <c r="Q59" s="59"/>
+      <c r="R59" s="59"/>
     </row>
     <row r="60" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1"/>
-      <c r="B60" s="40"/>
-      <c r="C60" s="41"/>
-      <c r="D60" s="42"/>
-      <c r="E60" s="43"/>
-      <c r="F60" s="44"/>
-      <c r="G60" s="45"/>
-      <c r="H60" s="44"/>
-      <c r="I60" s="45"/>
-      <c r="J60" s="44"/>
-      <c r="K60" s="45"/>
-      <c r="L60" s="45"/>
+      <c r="B60" s="91"/>
+      <c r="C60" s="92"/>
+      <c r="D60" s="93"/>
+      <c r="E60" s="94"/>
+      <c r="F60" s="95"/>
+      <c r="G60" s="96"/>
+      <c r="H60" s="95"/>
+      <c r="I60" s="96"/>
+      <c r="J60" s="95"/>
+      <c r="K60" s="96"/>
+      <c r="L60" s="96"/>
       <c r="M60" s="81" t="s">
         <v>5</v>
       </c>
@@ -5006,41 +5044,15 @@
         <f>SUM(P10:P59)</f>
         <v>31.379900000000003</v>
       </c>
-      <c r="Q60" s="83"/>
-      <c r="R60" s="84"/>
-    </row>
-    <row r="61" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="1"/>
-      <c r="B61" s="25"/>
-      <c r="C61" s="36"/>
-      <c r="D61" s="9"/>
-      <c r="E61" s="10"/>
-      <c r="F61" s="10"/>
-      <c r="G61" s="10"/>
-      <c r="H61" s="10"/>
-      <c r="I61" s="10"/>
-      <c r="J61" s="10"/>
-      <c r="K61" s="10"/>
-      <c r="L61" s="10"/>
-      <c r="M61" s="81" t="s">
-        <v>6</v>
-      </c>
-      <c r="N61" s="82"/>
-      <c r="O61" s="82"/>
-      <c r="P61" s="49">
-        <f>P60/2</f>
-        <v>15.689950000000001</v>
-      </c>
-      <c r="Q61" s="85"/>
-      <c r="R61" s="86"/>
+      <c r="Q60" s="97"/>
+      <c r="R60" s="98"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="4">
     <mergeCell ref="K1:R1"/>
     <mergeCell ref="R3:R8"/>
     <mergeCell ref="M60:O60"/>
-    <mergeCell ref="Q60:R61"/>
-    <mergeCell ref="M61:O61"/>
+    <mergeCell ref="Q60:R60"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="N10" r:id="rId1"/>
@@ -5104,7 +5116,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="3" max="3" width="13.5703125" customWidth="1"/>
     <col min="4" max="4" width="18.28515625" customWidth="1"/>
     <col min="5" max="5" width="29.85546875" customWidth="1"/>
     <col min="6" max="6" width="10.85546875" customWidth="1"/>

</xml_diff>

<commit_message>
#7 Component Price added in Client BOM
</commit_message>
<xml_diff>
--- a/Design Files/Xponent-tech/BOM/eSpark-BOM-Xponent-tech.xlsx
+++ b/Design Files/Xponent-tech/BOM/eSpark-BOM-Xponent-tech.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="1 Board" sheetId="3" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1644" uniqueCount="328">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1643" uniqueCount="328">
   <si>
     <t>Component list</t>
   </si>
@@ -4898,7 +4898,7 @@
       <c r="Q56" s="37"/>
       <c r="R56" s="59"/>
     </row>
-    <row r="57" spans="1:18" s="68" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:18" s="68" customFormat="1" ht="24" x14ac:dyDescent="0.25">
       <c r="A57" s="66"/>
       <c r="B57" s="47">
         <f t="shared" si="0"/>
@@ -4941,8 +4941,9 @@
       <c r="O57" s="38">
         <v>0.14399999999999999</v>
       </c>
-      <c r="P57" s="61" t="s">
-        <v>298</v>
+      <c r="P57" s="38">
+        <f>O57*M57</f>
+        <v>0.72</v>
       </c>
       <c r="Q57" s="60"/>
       <c r="R57" s="62"/>
@@ -5172,7 +5173,7 @@
       <c r="O62" s="97"/>
       <c r="P62" s="48">
         <f>SUM(P10:P61)</f>
-        <v>38.397500000000001</v>
+        <v>39.1175</v>
       </c>
       <c r="Q62" s="78"/>
       <c r="R62" s="91"/>

</xml_diff>